<commit_message>
Them tu dong hoa tao audio
</commit_message>
<xml_diff>
--- a/vocab_data.xlsx
+++ b/vocab_data.xlsx
@@ -502,6 +502,11 @@
       <c r="G2" t="n">
         <v>1</v>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>你.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -537,6 +542,11 @@
       <c r="G3" t="n">
         <v>1</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>您.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -572,6 +582,11 @@
       <c r="G4" t="n">
         <v>1</v>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>好.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -607,6 +622,11 @@
       <c r="G5" t="n">
         <v>1</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>大家好.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -642,6 +662,11 @@
       <c r="G6" t="n">
         <v>1</v>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>白.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -677,6 +702,11 @@
       <c r="G7" t="n">
         <v>1</v>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>大.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -712,6 +742,11 @@
       <c r="G8" t="n">
         <v>1</v>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>不.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -747,6 +782,11 @@
       <c r="G9" t="n">
         <v>1</v>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>女.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -782,6 +822,11 @@
       <c r="G10" t="n">
         <v>1</v>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>口红.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -817,6 +862,11 @@
       <c r="G11" t="n">
         <v>1</v>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>一.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -852,6 +902,11 @@
       <c r="G12" t="n">
         <v>1</v>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>五.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -887,6 +942,11 @@
       <c r="G13" t="n">
         <v>1</v>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>八.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -922,6 +982,11 @@
       <c r="G14" t="n">
         <v>1</v>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>难.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -957,6 +1022,11 @@
       <c r="G15" t="n">
         <v>1</v>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>忙.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -992,6 +1062,11 @@
       <c r="G16" t="n">
         <v>1</v>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>累.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1027,6 +1102,11 @@
       <c r="G17" t="n">
         <v>1</v>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>冷.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1062,6 +1142,11 @@
       <c r="G18" t="n">
         <v>1</v>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>红.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1097,6 +1182,11 @@
       <c r="G19" t="n">
         <v>1</v>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>高.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1132,6 +1222,11 @@
       <c r="G20" t="n">
         <v>1</v>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>真.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1167,6 +1262,11 @@
       <c r="G21" t="n">
         <v>1</v>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>太.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1202,6 +1302,11 @@
       <c r="G22" t="n">
         <v>1</v>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>很.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1237,6 +1342,11 @@
       <c r="G23" t="n">
         <v>1</v>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>爷爷.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1272,6 +1382,11 @@
       <c r="G24" t="n">
         <v>1</v>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>奶奶.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1307,6 +1422,11 @@
       <c r="G25" t="n">
         <v>1</v>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>外公.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1342,6 +1462,11 @@
       <c r="G26" t="n">
         <v>1</v>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>外婆.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1377,6 +1502,11 @@
       <c r="G27" t="n">
         <v>1</v>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>爸爸.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1412,6 +1542,11 @@
       <c r="G28" t="n">
         <v>1</v>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>妈妈.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1447,6 +1582,11 @@
       <c r="G29" t="n">
         <v>1</v>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>哥哥.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1482,6 +1622,11 @@
       <c r="G30" t="n">
         <v>1</v>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>姐姐.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1517,6 +1662,11 @@
       <c r="G31" t="n">
         <v>1</v>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>我.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1552,6 +1702,11 @@
       <c r="G32" t="n">
         <v>1</v>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>弟弟.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1587,6 +1742,11 @@
       <c r="G33" t="n">
         <v>1</v>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>妹妹.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1622,6 +1782,11 @@
       <c r="G34" t="n">
         <v>1</v>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>男.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1657,6 +1822,11 @@
       <c r="G35" t="n">
         <v>1</v>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>学习.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1692,6 +1862,11 @@
       <c r="G36" t="n">
         <v>1</v>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>英语.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1727,6 +1902,11 @@
       <c r="G37" t="n">
         <v>1</v>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>明天.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1762,6 +1942,11 @@
       <c r="G38" t="n">
         <v>1</v>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>见.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1797,6 +1982,11 @@
       <c r="G39" t="n">
         <v>1</v>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>一会儿见.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1832,6 +2022,11 @@
       <c r="G40" t="n">
         <v>1</v>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>后天见.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1867,6 +2062,11 @@
       <c r="G41" t="n">
         <v>1</v>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>再见.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1902,6 +2102,11 @@
       <c r="G42" t="n">
         <v>1</v>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>拜拜.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1937,6 +2142,11 @@
       <c r="G43" t="n">
         <v>1</v>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>外语.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1972,6 +2182,11 @@
       <c r="G44" t="n">
         <v>1</v>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>母语.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2007,6 +2222,11 @@
       <c r="G45" t="n">
         <v>1</v>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>越南语.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2042,6 +2262,11 @@
       <c r="G46" t="n">
         <v>1</v>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>邮局.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2077,6 +2302,11 @@
       <c r="G47" t="n">
         <v>1</v>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>寄信.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2112,6 +2342,11 @@
       <c r="G48" t="n">
         <v>1</v>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>寄明信片.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2147,6 +2382,11 @@
       <c r="G49" t="n">
         <v>1</v>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>寄包裹.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2182,6 +2422,11 @@
       <c r="G50" t="n">
         <v>1</v>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>拍照.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2217,6 +2462,11 @@
       <c r="G51" t="n">
         <v>1</v>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>打电话.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2252,6 +2502,11 @@
       <c r="G52" t="n">
         <v>2</v>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>爱.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2287,6 +2542,11 @@
       <c r="G53" t="n">
         <v>2</v>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>八.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2322,6 +2582,11 @@
       <c r="G54" t="n">
         <v>2</v>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>爸爸.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2357,6 +2622,11 @@
       <c r="G55" t="n">
         <v>2</v>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>杯子.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2392,6 +2662,11 @@
       <c r="G56" t="n">
         <v>2</v>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>北京.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2427,6 +2702,11 @@
       <c r="G57" t="n">
         <v>2</v>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>本.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2457,6 +2737,11 @@
       <c r="G58" t="n">
         <v>2</v>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>不客气.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2492,6 +2777,11 @@
       <c r="G59" t="n">
         <v>2</v>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>不.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2527,6 +2817,11 @@
       <c r="G60" t="n">
         <v>2</v>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>菜.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2562,6 +2857,11 @@
       <c r="G61" t="n">
         <v>2</v>
       </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>茶.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2597,6 +2897,11 @@
       <c r="G62" t="n">
         <v>2</v>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>吃.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2632,6 +2937,11 @@
       <c r="G63" t="n">
         <v>2</v>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>出租车.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2662,6 +2972,11 @@
       <c r="G64" t="n">
         <v>2</v>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>打电话.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2697,6 +3012,11 @@
       <c r="G65" t="n">
         <v>2</v>
       </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>大.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2732,6 +3052,11 @@
       <c r="G66" t="n">
         <v>2</v>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>的.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2767,6 +3092,11 @@
       <c r="G67" t="n">
         <v>2</v>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>点.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2802,6 +3132,11 @@
       <c r="G68" t="n">
         <v>2</v>
       </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>电脑.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2837,6 +3172,11 @@
       <c r="G69" t="n">
         <v>2</v>
       </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>电视.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2872,6 +3212,11 @@
       <c r="G70" t="n">
         <v>2</v>
       </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>电影.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2907,6 +3252,11 @@
       <c r="G71" t="n">
         <v>2</v>
       </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>东西.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2942,6 +3292,11 @@
       <c r="G72" t="n">
         <v>2</v>
       </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>都.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2977,6 +3332,11 @@
       <c r="G73" t="n">
         <v>2</v>
       </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>读.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3007,6 +3367,11 @@
       <c r="G74" t="n">
         <v>2</v>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>对不起.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3042,6 +3407,11 @@
       <c r="G75" t="n">
         <v>2</v>
       </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>多.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3077,6 +3447,11 @@
       <c r="G76" t="n">
         <v>2</v>
       </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>多少.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3112,6 +3487,11 @@
       <c r="G77" t="n">
         <v>2</v>
       </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>儿子.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3147,6 +3527,11 @@
       <c r="G78" t="n">
         <v>2</v>
       </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>二.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3182,6 +3567,11 @@
       <c r="G79" t="n">
         <v>2</v>
       </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>饭店.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3217,6 +3607,11 @@
       <c r="G80" t="n">
         <v>2</v>
       </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>飞机.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3252,6 +3647,11 @@
       <c r="G81" t="n">
         <v>2</v>
       </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>分钟.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3287,6 +3687,11 @@
       <c r="G82" t="n">
         <v>2</v>
       </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>高兴.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3322,6 +3727,11 @@
       <c r="G83" t="n">
         <v>2</v>
       </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>个.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3357,6 +3767,11 @@
       <c r="G84" t="n">
         <v>2</v>
       </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>工作.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3392,6 +3807,11 @@
       <c r="G85" t="n">
         <v>2</v>
       </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>汉语.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3427,6 +3847,11 @@
       <c r="G86" t="n">
         <v>2</v>
       </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>好.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3462,6 +3887,11 @@
       <c r="G87" t="n">
         <v>2</v>
       </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>号.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3497,6 +3927,11 @@
       <c r="G88" t="n">
         <v>2</v>
       </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>喝.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3532,6 +3967,11 @@
       <c r="G89" t="n">
         <v>2</v>
       </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>和.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3567,6 +4007,11 @@
       <c r="G90" t="n">
         <v>2</v>
       </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>很.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3602,6 +4047,11 @@
       <c r="G91" t="n">
         <v>2</v>
       </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>后面.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3637,6 +4087,11 @@
       <c r="G92" t="n">
         <v>2</v>
       </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>回.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3672,6 +4127,11 @@
       <c r="G93" t="n">
         <v>2</v>
       </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>会.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3707,6 +4167,11 @@
       <c r="G94" t="n">
         <v>2</v>
       </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>几.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3742,6 +4207,11 @@
       <c r="G95" t="n">
         <v>2</v>
       </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>家.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3777,6 +4247,11 @@
       <c r="G96" t="n">
         <v>2</v>
       </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>叫.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3812,6 +4287,11 @@
       <c r="G97" t="n">
         <v>2</v>
       </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>今天.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3847,6 +4327,11 @@
       <c r="G98" t="n">
         <v>2</v>
       </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>九.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3882,6 +4367,11 @@
       <c r="G99" t="n">
         <v>2</v>
       </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>开.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3917,6 +4407,11 @@
       <c r="G100" t="n">
         <v>2</v>
       </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>看.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3952,6 +4447,11 @@
       <c r="G101" t="n">
         <v>2</v>
       </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>看见.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3987,6 +4487,11 @@
       <c r="G102" t="n">
         <v>2</v>
       </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>块.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4022,6 +4527,11 @@
       <c r="G103" t="n">
         <v>2</v>
       </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>来.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4057,6 +4567,11 @@
       <c r="G104" t="n">
         <v>2</v>
       </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>老师.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4092,6 +4607,11 @@
       <c r="G105" t="n">
         <v>2</v>
       </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>了.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4127,6 +4647,11 @@
       <c r="G106" t="n">
         <v>2</v>
       </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>冷.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4162,6 +4687,11 @@
       <c r="G107" t="n">
         <v>2</v>
       </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>里.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4197,6 +4727,11 @@
       <c r="G108" t="n">
         <v>2</v>
       </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>零.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4232,6 +4767,11 @@
       <c r="G109" t="n">
         <v>2</v>
       </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>六.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4267,6 +4807,11 @@
       <c r="G110" t="n">
         <v>2</v>
       </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>妈妈.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4302,6 +4847,11 @@
       <c r="G111" t="n">
         <v>2</v>
       </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>吗.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4337,6 +4887,11 @@
       <c r="G112" t="n">
         <v>2</v>
       </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>买.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4367,6 +4922,11 @@
       <c r="G113" t="n">
         <v>2</v>
       </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>没关系.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4402,6 +4962,11 @@
       <c r="G114" t="n">
         <v>2</v>
       </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>没有.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4437,6 +5002,11 @@
       <c r="G115" t="n">
         <v>2</v>
       </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>米饭.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4472,6 +5042,11 @@
       <c r="G116" t="n">
         <v>2</v>
       </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>明天.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4507,6 +5082,11 @@
       <c r="G117" t="n">
         <v>2</v>
       </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>名字.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4542,6 +5122,11 @@
       <c r="G118" t="n">
         <v>2</v>
       </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>哪.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4577,6 +5162,11 @@
       <c r="G119" t="n">
         <v>2</v>
       </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>哪儿.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4612,6 +5202,11 @@
       <c r="G120" t="n">
         <v>2</v>
       </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>那_那儿.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4647,6 +5242,11 @@
       <c r="G121" t="n">
         <v>2</v>
       </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>呢.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4682,6 +5282,11 @@
       <c r="G122" t="n">
         <v>2</v>
       </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>能.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4717,6 +5322,11 @@
       <c r="G123" t="n">
         <v>2</v>
       </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>你.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4752,6 +5362,11 @@
       <c r="G124" t="n">
         <v>2</v>
       </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>年.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4787,6 +5402,11 @@
       <c r="G125" t="n">
         <v>2</v>
       </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>女儿.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4822,6 +5442,11 @@
       <c r="G126" t="n">
         <v>2</v>
       </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>朋友.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4857,6 +5482,11 @@
       <c r="G127" t="n">
         <v>2</v>
       </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>漂亮.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4892,6 +5522,11 @@
       <c r="G128" t="n">
         <v>2</v>
       </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>苹果.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4927,6 +5562,11 @@
       <c r="G129" t="n">
         <v>2</v>
       </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>七.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4962,6 +5602,11 @@
       <c r="G130" t="n">
         <v>2</v>
       </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>钱.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4997,6 +5642,11 @@
       <c r="G131" t="n">
         <v>2</v>
       </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>前面.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5032,6 +5682,11 @@
       <c r="G132" t="n">
         <v>2</v>
       </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>请.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5067,6 +5722,11 @@
       <c r="G133" t="n">
         <v>2</v>
       </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>去.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5102,6 +5762,11 @@
       <c r="G134" t="n">
         <v>2</v>
       </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>热.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5137,6 +5802,11 @@
       <c r="G135" t="n">
         <v>2</v>
       </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>人.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5172,6 +5842,11 @@
       <c r="G136" t="n">
         <v>2</v>
       </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>认识.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5207,6 +5882,11 @@
       <c r="G137" t="n">
         <v>2</v>
       </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>三.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5242,6 +5922,11 @@
       <c r="G138" t="n">
         <v>2</v>
       </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>商店.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5277,6 +5962,11 @@
       <c r="G139" t="n">
         <v>2</v>
       </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>上.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5312,6 +6002,11 @@
       <c r="G140" t="n">
         <v>2</v>
       </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>上午.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5347,6 +6042,11 @@
       <c r="G141" t="n">
         <v>2</v>
       </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>少.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5382,6 +6082,11 @@
       <c r="G142" t="n">
         <v>2</v>
       </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>谁.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5417,6 +6122,11 @@
       <c r="G143" t="n">
         <v>2</v>
       </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>什么.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5452,6 +6162,11 @@
       <c r="G144" t="n">
         <v>2</v>
       </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>十.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5487,6 +6202,11 @@
       <c r="G145" t="n">
         <v>2</v>
       </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>时候.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5522,6 +6242,11 @@
       <c r="G146" t="n">
         <v>2</v>
       </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>是.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5557,6 +6282,11 @@
       <c r="G147" t="n">
         <v>2</v>
       </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>书.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5592,6 +6322,11 @@
       <c r="G148" t="n">
         <v>2</v>
       </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>水.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5627,6 +6362,11 @@
       <c r="G149" t="n">
         <v>2</v>
       </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>水果.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5662,6 +6402,11 @@
       <c r="G150" t="n">
         <v>2</v>
       </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>睡觉.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5697,6 +6442,11 @@
       <c r="G151" t="n">
         <v>2</v>
       </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>说.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5732,6 +6482,11 @@
       <c r="G152" t="n">
         <v>2</v>
       </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>说话.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5767,6 +6522,11 @@
       <c r="G153" t="n">
         <v>2</v>
       </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>四.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5802,6 +6562,11 @@
       <c r="G154" t="n">
         <v>2</v>
       </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>岁.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5837,6 +6602,11 @@
       <c r="G155" t="n">
         <v>2</v>
       </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>他.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5872,6 +6642,11 @@
       <c r="G156" t="n">
         <v>2</v>
       </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>她.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5907,6 +6682,11 @@
       <c r="G157" t="n">
         <v>2</v>
       </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>太.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5942,6 +6722,11 @@
       <c r="G158" t="n">
         <v>2</v>
       </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>天气.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5977,6 +6762,11 @@
       <c r="G159" t="n">
         <v>2</v>
       </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>听.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6012,6 +6802,11 @@
       <c r="G160" t="n">
         <v>2</v>
       </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>同学.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6047,6 +6842,11 @@
       <c r="G161" t="n">
         <v>2</v>
       </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>喂.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6082,6 +6882,11 @@
       <c r="G162" t="n">
         <v>2</v>
       </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>我.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6117,6 +6922,11 @@
       <c r="G163" t="n">
         <v>2</v>
       </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>我们.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -6152,6 +6962,11 @@
       <c r="G164" t="n">
         <v>2</v>
       </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>五.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6187,6 +7002,11 @@
       <c r="G165" t="n">
         <v>2</v>
       </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>喜欢.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -6222,6 +7042,11 @@
       <c r="G166" t="n">
         <v>2</v>
       </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>下.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -6257,6 +7082,11 @@
       <c r="G167" t="n">
         <v>2</v>
       </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>下午.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -6292,6 +7122,11 @@
       <c r="G168" t="n">
         <v>2</v>
       </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>下雨.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -6327,6 +7162,11 @@
       <c r="G169" t="n">
         <v>2</v>
       </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>先生.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -6362,6 +7202,11 @@
       <c r="G170" t="n">
         <v>2</v>
       </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>现在.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -6397,6 +7242,11 @@
       <c r="G171" t="n">
         <v>2</v>
       </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>想.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6432,6 +7282,11 @@
       <c r="G172" t="n">
         <v>2</v>
       </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>小.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -6467,6 +7322,11 @@
       <c r="G173" t="n">
         <v>2</v>
       </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>小姐.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -6502,6 +7362,11 @@
       <c r="G174" t="n">
         <v>2</v>
       </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>些.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -6537,6 +7402,11 @@
       <c r="G175" t="n">
         <v>2</v>
       </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>写.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -6572,6 +7442,11 @@
       <c r="G176" t="n">
         <v>2</v>
       </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>谢谢.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -6607,6 +7482,11 @@
       <c r="G177" t="n">
         <v>2</v>
       </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>星期.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6642,6 +7522,11 @@
       <c r="G178" t="n">
         <v>2</v>
       </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>学生.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6677,6 +7562,11 @@
       <c r="G179" t="n">
         <v>2</v>
       </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>学习.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6712,6 +7602,11 @@
       <c r="G180" t="n">
         <v>2</v>
       </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>学校.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6747,6 +7642,11 @@
       <c r="G181" t="n">
         <v>2</v>
       </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>一.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -6782,6 +7682,11 @@
       <c r="G182" t="n">
         <v>2</v>
       </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>一点儿.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6817,6 +7722,11 @@
       <c r="G183" t="n">
         <v>2</v>
       </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>衣服.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -6852,6 +7762,11 @@
       <c r="G184" t="n">
         <v>2</v>
       </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>医生.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -6887,6 +7802,11 @@
       <c r="G185" t="n">
         <v>2</v>
       </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>医院.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6922,6 +7842,11 @@
       <c r="G186" t="n">
         <v>2</v>
       </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>椅子.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6957,6 +7882,11 @@
       <c r="G187" t="n">
         <v>2</v>
       </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>有.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6992,6 +7922,11 @@
       <c r="G188" t="n">
         <v>2</v>
       </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>月.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -7022,6 +7957,11 @@
       <c r="G189" t="n">
         <v>2</v>
       </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>再见.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -7057,6 +7997,11 @@
       <c r="G190" t="n">
         <v>2</v>
       </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>在.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -7092,6 +8037,11 @@
       <c r="G191" t="n">
         <v>2</v>
       </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>怎么.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -7127,6 +8077,11 @@
       <c r="G192" t="n">
         <v>2</v>
       </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>怎么样.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -7162,6 +8117,11 @@
       <c r="G193" t="n">
         <v>2</v>
       </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>这_这儿.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -7197,6 +8157,11 @@
       <c r="G194" t="n">
         <v>2</v>
       </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>中国.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -7232,6 +8197,11 @@
       <c r="G195" t="n">
         <v>2</v>
       </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>中午.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -7267,6 +8237,11 @@
       <c r="G196" t="n">
         <v>2</v>
       </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>住.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -7302,6 +8277,11 @@
       <c r="G197" t="n">
         <v>2</v>
       </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>桌子.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -7337,6 +8317,11 @@
       <c r="G198" t="n">
         <v>2</v>
       </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>字.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -7372,6 +8357,11 @@
       <c r="G199" t="n">
         <v>2</v>
       </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>昨天.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -7407,6 +8397,11 @@
       <c r="G200" t="n">
         <v>2</v>
       </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>坐.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -7442,6 +8437,11 @@
       <c r="G201" t="n">
         <v>2</v>
       </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>做.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -7477,6 +8477,11 @@
       <c r="G202" t="n">
         <v>2</v>
       </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>吧.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -7512,6 +8517,11 @@
       <c r="G203" t="n">
         <v>2</v>
       </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>白.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -7547,6 +8557,11 @@
       <c r="G204" t="n">
         <v>2</v>
       </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>百.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -7582,6 +8597,11 @@
       <c r="G205" t="n">
         <v>2</v>
       </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>帮助.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -7617,6 +8637,11 @@
       <c r="G206" t="n">
         <v>2</v>
       </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>报纸.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -7652,6 +8677,11 @@
       <c r="G207" t="n">
         <v>2</v>
       </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>比.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -7687,6 +8717,11 @@
       <c r="G208" t="n">
         <v>2</v>
       </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>别.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -7722,6 +8757,11 @@
       <c r="G209" t="n">
         <v>2</v>
       </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>长.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -7757,6 +8797,11 @@
       <c r="G210" t="n">
         <v>2</v>
       </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>唱歌.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -7792,6 +8837,11 @@
       <c r="G211" t="n">
         <v>2</v>
       </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>出.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -7827,6 +8877,11 @@
       <c r="G212" t="n">
         <v>2</v>
       </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>穿.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -7862,6 +8917,11 @@
       <c r="G213" t="n">
         <v>2</v>
       </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>次.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -7897,6 +8957,11 @@
       <c r="G214" t="n">
         <v>2</v>
       </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>从.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -7932,6 +8997,11 @@
       <c r="G215" t="n">
         <v>2</v>
       </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>错.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -7962,6 +9032,11 @@
       <c r="G216" t="n">
         <v>2</v>
       </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>打篮球.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -7997,6 +9072,11 @@
       <c r="G217" t="n">
         <v>2</v>
       </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>大家.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -8032,6 +9112,11 @@
       <c r="G218" t="n">
         <v>2</v>
       </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>到.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -8067,6 +9152,11 @@
       <c r="G219" t="n">
         <v>2</v>
       </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>得.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -8102,6 +9192,11 @@
       <c r="G220" t="n">
         <v>2</v>
       </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>等.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -8137,6 +9232,11 @@
       <c r="G221" t="n">
         <v>2</v>
       </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>弟弟.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -8172,6 +9272,11 @@
       <c r="G222" t="n">
         <v>2</v>
       </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>第一.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -8207,6 +9312,11 @@
       <c r="G223" t="n">
         <v>2</v>
       </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>懂.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -8242,6 +9352,11 @@
       <c r="G224" t="n">
         <v>2</v>
       </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>对.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -8277,6 +9392,11 @@
       <c r="G225" t="n">
         <v>2</v>
       </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>对.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -8312,6 +9432,11 @@
       <c r="G226" t="n">
         <v>2</v>
       </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>房间.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -8347,6 +9472,11 @@
       <c r="G227" t="n">
         <v>2</v>
       </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>非常.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -8382,6 +9512,11 @@
       <c r="G228" t="n">
         <v>2</v>
       </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>服务员.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -8417,6 +9552,11 @@
       <c r="G229" t="n">
         <v>2</v>
       </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>高.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -8452,6 +9592,11 @@
       <c r="G230" t="n">
         <v>2</v>
       </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>告诉.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -8487,6 +9632,11 @@
       <c r="G231" t="n">
         <v>2</v>
       </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>哥哥.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -8522,6 +9672,11 @@
       <c r="G232" t="n">
         <v>2</v>
       </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>给.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -8557,6 +9712,11 @@
       <c r="G233" t="n">
         <v>2</v>
       </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>公共汽车.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -8592,6 +9752,11 @@
       <c r="G234" t="n">
         <v>2</v>
       </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>公司.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -8627,6 +9792,11 @@
       <c r="G235" t="n">
         <v>2</v>
       </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>狗.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -8662,6 +9832,11 @@
       <c r="G236" t="n">
         <v>2</v>
       </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>贵.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -8697,6 +9872,11 @@
       <c r="G237" t="n">
         <v>2</v>
       </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>过.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -8732,6 +9912,11 @@
       <c r="G238" t="n">
         <v>2</v>
       </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>还.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -8767,6 +9952,11 @@
       <c r="G239" t="n">
         <v>2</v>
       </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>孩子.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -8802,6 +9992,11 @@
       <c r="G240" t="n">
         <v>2</v>
       </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>好吃.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -8837,6 +10032,11 @@
       <c r="G241" t="n">
         <v>2</v>
       </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>黑.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -8872,6 +10072,11 @@
       <c r="G242" t="n">
         <v>2</v>
       </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>红.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -8907,6 +10112,11 @@
       <c r="G243" t="n">
         <v>2</v>
       </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>欢迎.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -8942,6 +10152,11 @@
       <c r="G244" t="n">
         <v>2</v>
       </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>回答.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -8977,6 +10192,11 @@
       <c r="G245" t="n">
         <v>2</v>
       </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>火车站.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -9012,6 +10232,11 @@
       <c r="G246" t="n">
         <v>2</v>
       </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>机场.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -9047,6 +10272,11 @@
       <c r="G247" t="n">
         <v>2</v>
       </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>鸡蛋.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -9082,6 +10312,11 @@
       <c r="G248" t="n">
         <v>2</v>
       </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>件.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -9117,6 +10352,11 @@
       <c r="G249" t="n">
         <v>2</v>
       </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>教室.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -9152,6 +10392,11 @@
       <c r="G250" t="n">
         <v>2</v>
       </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>姐姐.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -9187,6 +10432,11 @@
       <c r="G251" t="n">
         <v>2</v>
       </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>介绍.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -9222,6 +10472,11 @@
       <c r="G252" t="n">
         <v>2</v>
       </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>进.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -9257,6 +10512,11 @@
       <c r="G253" t="n">
         <v>2</v>
       </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>近.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -9292,6 +10552,11 @@
       <c r="G254" t="n">
         <v>2</v>
       </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>就.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -9327,6 +10592,11 @@
       <c r="G255" t="n">
         <v>2</v>
       </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>觉得.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -9362,6 +10632,11 @@
       <c r="G256" t="n">
         <v>2</v>
       </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>咖啡.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -9397,6 +10672,11 @@
       <c r="G257" t="n">
         <v>2</v>
       </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>开始.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -9432,6 +10712,11 @@
       <c r="G258" t="n">
         <v>2</v>
       </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>考试.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -9467,6 +10752,11 @@
       <c r="G259" t="n">
         <v>2</v>
       </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>可能.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -9502,6 +10792,11 @@
       <c r="G260" t="n">
         <v>2</v>
       </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>可以.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -9537,6 +10832,11 @@
       <c r="G261" t="n">
         <v>2</v>
       </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>课.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -9572,6 +10872,11 @@
       <c r="G262" t="n">
         <v>2</v>
       </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>快.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -9607,6 +10912,11 @@
       <c r="G263" t="n">
         <v>2</v>
       </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>快乐.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -9642,6 +10952,11 @@
       <c r="G264" t="n">
         <v>2</v>
       </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>累.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -9677,6 +10992,11 @@
       <c r="G265" t="n">
         <v>2</v>
       </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>离.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -9712,6 +11032,11 @@
       <c r="G266" t="n">
         <v>2</v>
       </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>两.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -9747,6 +11072,11 @@
       <c r="G267" t="n">
         <v>2</v>
       </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>路.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -9782,6 +11112,11 @@
       <c r="G268" t="n">
         <v>2</v>
       </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>旅游.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -9817,6 +11152,11 @@
       <c r="G269" t="n">
         <v>2</v>
       </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>卖.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -9852,6 +11192,11 @@
       <c r="G270" t="n">
         <v>2</v>
       </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>慢.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -9887,6 +11232,11 @@
       <c r="G271" t="n">
         <v>2</v>
       </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>忙.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -9922,6 +11272,11 @@
       <c r="G272" t="n">
         <v>2</v>
       </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>猫.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -9957,6 +11312,11 @@
       <c r="G273" t="n">
         <v>2</v>
       </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>每.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -9992,6 +11352,11 @@
       <c r="G274" t="n">
         <v>2</v>
       </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>妹妹.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -10027,6 +11392,11 @@
       <c r="G275" t="n">
         <v>2</v>
       </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>门.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -10062,6 +11432,11 @@
       <c r="G276" t="n">
         <v>2</v>
       </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>男.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -10097,6 +11472,11 @@
       <c r="G277" t="n">
         <v>2</v>
       </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>您.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -10132,6 +11512,11 @@
       <c r="G278" t="n">
         <v>2</v>
       </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>牛奶.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -10167,6 +11552,11 @@
       <c r="G279" t="n">
         <v>2</v>
       </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>女.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -10202,6 +11592,11 @@
       <c r="G280" t="n">
         <v>2</v>
       </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>旁边.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -10237,6 +11632,11 @@
       <c r="G281" t="n">
         <v>2</v>
       </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>跑步.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -10272,6 +11672,11 @@
       <c r="G282" t="n">
         <v>2</v>
       </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>便宜.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -10307,6 +11712,11 @@
       <c r="G283" t="n">
         <v>2</v>
       </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>票.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -10342,6 +11752,11 @@
       <c r="G284" t="n">
         <v>2</v>
       </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>妻子.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -10377,6 +11792,11 @@
       <c r="G285" t="n">
         <v>2</v>
       </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>起床.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -10412,6 +11832,11 @@
       <c r="G286" t="n">
         <v>2</v>
       </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>千.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -10447,6 +11872,11 @@
       <c r="G287" t="n">
         <v>2</v>
       </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>铅笔.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -10482,6 +11912,11 @@
       <c r="G288" t="n">
         <v>2</v>
       </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>晴.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -10517,6 +11952,11 @@
       <c r="G289" t="n">
         <v>2</v>
       </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>去年.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -10552,6 +11992,11 @@
       <c r="G290" t="n">
         <v>2</v>
       </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>让.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -10587,6 +12032,11 @@
       <c r="G291" t="n">
         <v>2</v>
       </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>日.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -10622,6 +12072,11 @@
       <c r="G292" t="n">
         <v>2</v>
       </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>上班.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -10657,6 +12112,11 @@
       <c r="G293" t="n">
         <v>2</v>
       </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>身体.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -10692,6 +12152,11 @@
       <c r="G294" t="n">
         <v>2</v>
       </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>生病.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -10727,6 +12192,11 @@
       <c r="G295" t="n">
         <v>2</v>
       </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>生日.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -10762,6 +12232,11 @@
       <c r="G296" t="n">
         <v>2</v>
       </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>时间.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -10797,6 +12272,11 @@
       <c r="G297" t="n">
         <v>2</v>
       </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>事情.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -10832,6 +12312,11 @@
       <c r="G298" t="n">
         <v>2</v>
       </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>手表.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -10867,6 +12352,11 @@
       <c r="G299" t="n">
         <v>2</v>
       </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>手机.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -10902,6 +12392,11 @@
       <c r="G300" t="n">
         <v>2</v>
       </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>送.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -10937,6 +12432,11 @@
       <c r="G301" t="n">
         <v>2</v>
       </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>虽然_但是.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -10972,6 +12472,11 @@
       <c r="G302" t="n">
         <v>2</v>
       </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>它.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -11002,6 +12507,11 @@
       <c r="G303" t="n">
         <v>2</v>
       </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>踢足球.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -11037,6 +12547,11 @@
       <c r="G304" t="n">
         <v>2</v>
       </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>题.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -11072,6 +12587,11 @@
       <c r="G305" t="n">
         <v>2</v>
       </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>跳舞.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -11107,6 +12627,11 @@
       <c r="G306" t="n">
         <v>2</v>
       </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>外.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -11142,6 +12667,11 @@
       <c r="G307" t="n">
         <v>2</v>
       </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>完.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -11177,6 +12707,11 @@
       <c r="G308" t="n">
         <v>2</v>
       </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>玩.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -11212,6 +12747,11 @@
       <c r="G309" t="n">
         <v>2</v>
       </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>晚上.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -11247,6 +12787,11 @@
       <c r="G310" t="n">
         <v>2</v>
       </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>为什么.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -11282,6 +12827,11 @@
       <c r="G311" t="n">
         <v>2</v>
       </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>问.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -11317,6 +12867,11 @@
       <c r="G312" t="n">
         <v>2</v>
       </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>问题.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -11352,6 +12907,11 @@
       <c r="G313" t="n">
         <v>2</v>
       </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>西瓜.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -11387,6 +12947,11 @@
       <c r="G314" t="n">
         <v>2</v>
       </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>希望.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -11422,6 +12987,11 @@
       <c r="G315" t="n">
         <v>2</v>
       </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>洗.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -11457,6 +13027,11 @@
       <c r="G316" t="n">
         <v>2</v>
       </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>小时.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -11492,6 +13067,11 @@
       <c r="G317" t="n">
         <v>2</v>
       </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>笑.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -11527,6 +13107,11 @@
       <c r="G318" t="n">
         <v>2</v>
       </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>新.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -11562,6 +13147,11 @@
       <c r="G319" t="n">
         <v>2</v>
       </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>姓.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -11597,6 +13187,11 @@
       <c r="G320" t="n">
         <v>2</v>
       </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>休息.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -11632,6 +13227,11 @@
       <c r="G321" t="n">
         <v>2</v>
       </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>雪.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -11667,6 +13267,11 @@
       <c r="G322" t="n">
         <v>2</v>
       </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>颜色.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -11702,6 +13307,11 @@
       <c r="G323" t="n">
         <v>2</v>
       </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>眼睛.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -11737,6 +13347,11 @@
       <c r="G324" t="n">
         <v>2</v>
       </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>羊肉.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -11772,6 +13387,11 @@
       <c r="G325" t="n">
         <v>2</v>
       </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>药.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -11807,6 +13427,11 @@
       <c r="G326" t="n">
         <v>2</v>
       </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>要.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -11842,6 +13467,11 @@
       <c r="G327" t="n">
         <v>2</v>
       </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>也.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -11877,6 +13507,11 @@
       <c r="G328" t="n">
         <v>2</v>
       </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>一下.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -11912,6 +13547,11 @@
       <c r="G329" t="n">
         <v>2</v>
       </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>一起.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -11947,6 +13587,11 @@
       <c r="G330" t="n">
         <v>2</v>
       </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>已经.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -11982,6 +13627,11 @@
       <c r="G331" t="n">
         <v>2</v>
       </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>意思.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -12017,6 +13667,11 @@
       <c r="G332" t="n">
         <v>2</v>
       </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>因为_所以.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -12052,6 +13707,11 @@
       <c r="G333" t="n">
         <v>2</v>
       </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>阴.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -12087,6 +13747,11 @@
       <c r="G334" t="n">
         <v>2</v>
       </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>游泳.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -12122,6 +13787,11 @@
       <c r="G335" t="n">
         <v>2</v>
       </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>右边.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -12157,6 +13827,11 @@
       <c r="G336" t="n">
         <v>2</v>
       </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>鱼.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -12192,6 +13867,11 @@
       <c r="G337" t="n">
         <v>2</v>
       </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>远.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -12227,6 +13907,11 @@
       <c r="G338" t="n">
         <v>2</v>
       </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>运动.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -12262,6 +13947,11 @@
       <c r="G339" t="n">
         <v>2</v>
       </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>再.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -12297,6 +13987,11 @@
       <c r="G340" t="n">
         <v>2</v>
       </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>早上.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -12332,6 +14027,11 @@
       <c r="G341" t="n">
         <v>2</v>
       </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>丈夫.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -12367,6 +14067,11 @@
       <c r="G342" t="n">
         <v>2</v>
       </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>找.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -12402,6 +14107,11 @@
       <c r="G343" t="n">
         <v>2</v>
       </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>着.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -12437,6 +14147,11 @@
       <c r="G344" t="n">
         <v>2</v>
       </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>真.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -12472,6 +14187,11 @@
       <c r="G345" t="n">
         <v>2</v>
       </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>正在.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -12507,6 +14227,11 @@
       <c r="G346" t="n">
         <v>2</v>
       </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>知道.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -12542,6 +14267,11 @@
       <c r="G347" t="n">
         <v>2</v>
       </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>准备.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -12577,6 +14307,11 @@
       <c r="G348" t="n">
         <v>2</v>
       </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>自行车.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -12612,6 +14347,11 @@
       <c r="G349" t="n">
         <v>2</v>
       </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>走.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -12647,6 +14387,11 @@
       <c r="G350" t="n">
         <v>2</v>
       </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>最.mp3</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -12681,6 +14426,11 @@
       </c>
       <c r="G351" t="n">
         <v>2</v>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>左边.mp3</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tu dong cap nhat vocab.json va audio tu Excel
</commit_message>
<xml_diff>
--- a/vocab_data.xlsx
+++ b/vocab_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tu vung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tu vung" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>